<commit_message>
Extend dataset for margin, renegotiation and budget scenarios
- Generator: customer piece prices (contract Annex A + SAP price
  conditions with a stale 2025 price), product standard costs,
  renegotiation clauses (hardship, price review, price-down waiver,
  extraordinary review, cost sharing, meet-competition, volume rebate,
  renewal), RFQ responses, negotiation log, Keystone renewal offer and an
  FY2027 budget built on June 2026 prices; latest forecast now diverges
  from budget volumes
- Ingestion: SAP customer master and price conditions, standard costs on
  products, RFQs as price quotes, negotiations, plans and plan_lines
- Extraction: levers, piece prices and offer details; SAP vs contract
  piece-price cross-check; scripts/check_extraction.py (110/110 correct)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/sales/forecast_US_plant_2026-10.xlsx
+++ b/data/raw/sales/forecast_US_plant_2026-10.xlsx
@@ -464,7 +464,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1990</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="3">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1996</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="4">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1586</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="5">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1833</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="6">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2292</v>
+        <v>1948</v>
       </c>
     </row>
     <row r="7">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2516</v>
+        <v>2139</v>
       </c>
     </row>
     <row r="8">
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2382</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="9">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2270</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="10">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1969</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="11">
@@ -644,7 +644,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1412</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="12">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1733</v>
+        <v>1473</v>
       </c>
     </row>
     <row r="13">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2125</v>
+        <v>1807</v>
       </c>
     </row>
     <row r="14">
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>784</v>
+        <v>667</v>
       </c>
     </row>
     <row r="15">
@@ -724,7 +724,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>791</v>
+        <v>672</v>
       </c>
     </row>
     <row r="16">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>621</v>
+        <v>528</v>
       </c>
     </row>
     <row r="17">
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>725</v>
+        <v>617</v>
       </c>
     </row>
     <row r="18">
@@ -784,7 +784,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>778</v>
+        <v>661</v>
       </c>
     </row>
     <row r="19">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>811</v>
+        <v>690</v>
       </c>
     </row>
     <row r="20">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>799</v>
+        <v>679</v>
       </c>
     </row>
     <row r="21">
@@ -844,7 +844,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>739</v>
+        <v>628</v>
       </c>
     </row>
     <row r="22">
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>722</v>
+        <v>614</v>
       </c>
     </row>
     <row r="23">
@@ -884,7 +884,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>536</v>
+        <v>456</v>
       </c>
     </row>
     <row r="24">
@@ -904,7 +904,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>631</v>
+        <v>536</v>
       </c>
     </row>
     <row r="25">
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>764</v>
+        <v>650</v>
       </c>
     </row>
     <row r="26">
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1288</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="27">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1334</v>
+        <v>1134</v>
       </c>
     </row>
     <row r="28">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1037</v>
+        <v>881</v>
       </c>
     </row>
     <row r="29">
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1058</v>
+        <v>899</v>
       </c>
     </row>
     <row r="30">
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1160</v>
+        <v>986</v>
       </c>
     </row>
     <row r="31">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1427</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="32">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1417</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="33">
@@ -1084,7 +1084,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1352</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="34">
@@ -1104,7 +1104,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1233</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="35">
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>947</v>
+        <v>805</v>
       </c>
     </row>
     <row r="36">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1120</v>
+        <v>952</v>
       </c>
     </row>
     <row r="37">
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1418</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="38">

</xml_diff>